<commit_message>
Add cancelled cheque and fill bank details in Mayfair vendor form
Fill bank name, account number, IFSC and bank address from the Axis Bank
cancelled cheque, tick Current Account, and update the checklist.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UbJaKorh4mZTkXzSUC4k7b
</commit_message>
<xml_diff>
--- a/Mayfair Docs/Filled - Joes Jyoti Services/Vendor Registration Form - Joes Jyoti Services.xlsx
+++ b/Mayfair Docs/Filled - Joes Jyoti Services/Vendor Registration Form - Joes Jyoti Services.xlsx
@@ -613,7 +613,7 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp9.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" lockText="1" noThreeD="1"/>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2322,13 +2322,21 @@
       <c r="A32" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="B32" s="9"/>
+      <c r="B32" s="9" t="inlineStr">
+        <is>
+          <t>Axis Bank Ltd</t>
+        </is>
+      </c>
     </row>
     <row r="33" spans="1:2" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="B33" s="22"/>
+      <c r="B33" s="22" t="inlineStr">
+        <is>
+          <t>919020019694374</t>
+        </is>
+      </c>
     </row>
     <row r="34" spans="1:2" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="10" t="s">
@@ -2340,13 +2348,21 @@
       <c r="A35" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="B35" s="9"/>
+      <c r="B35" s="9" t="inlineStr">
+        <is>
+          <t>UTIB0000381</t>
+        </is>
+      </c>
     </row>
     <row r="36" spans="1:2" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="B36" s="9"/>
+      <c r="B36" s="9" t="inlineStr">
+        <is>
+          <t>Axis Bank Ltd, Chandrasekharpur, Bhubaneswar, Odisha - 751016</t>
+        </is>
+      </c>
     </row>
     <row r="37" spans="1:2" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="8" t="s">

</xml_diff>

<commit_message>
Add renewed FSSAI licence and Udyam certificate, update vendor pack
Fill MSME/Udyam details in the vendor form, drop the MSME non-registration
declaration since the company is Udyam registered, and update the checklist
for the renewed FSSAI licence.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UbJaKorh4mZTkXzSUC4k7b
</commit_message>
<xml_diff>
--- a/Mayfair Docs/Filled - Joes Jyoti Services/Vendor Registration Form - Joes Jyoti Services.xlsx
+++ b/Mayfair Docs/Filled - Joes Jyoti Services/Vendor Registration Form - Joes Jyoti Services.xlsx
@@ -2430,7 +2430,11 @@
       <c r="A44" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="B44" s="9"/>
+      <c r="B44" s="9" t="inlineStr">
+        <is>
+          <t>UDYAM-OD-19-0057563</t>
+        </is>
+      </c>
     </row>
     <row r="45" spans="1:2" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="10" t="s">
@@ -2458,13 +2462,21 @@
       <c r="A48" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B48" s="9"/>
+      <c r="B48" s="9" t="inlineStr">
+        <is>
+          <t>Yes - Udyam Registration No. UDYAM-OD-19-0057563 (Micro enterprise)</t>
+        </is>
+      </c>
     </row>
     <row r="49" spans="1:18" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="B49" s="9"/>
+      <c r="B49" s="9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="50" spans="1:18" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="33" t="s">

</xml_diff>